<commit_message>
Reconstruct proven own-break outcomes from surviving rack history
</commit_message>
<xml_diff>
--- a/docs/examples/federal-96-linked-doubles.xlsx
+++ b/docs/examples/federal-96-linked-doubles.xlsx
@@ -263,15 +263,11 @@
           <t xml:space="preserve">Break and win</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="B13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
@@ -280,15 +276,11 @@
           <t xml:space="preserve">Break and lose</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—</t>
-        </is>
+      <c r="B14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>